<commit_message>
chore: unsaved excel changes
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/11-wastewater.xlsx
+++ b/packages/calculators/src/modules/test/11-wastewater.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD013870-5A16-734A-9E9D-B0650BC2CABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6A69E8-7FBF-B24A-9A69-8910D0934DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6820" yWindow="-21600" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="11.1" sheetId="1" r:id="rId1"/>

</xml_diff>